<commit_message>
version actualiza fechas de agentes
</commit_message>
<xml_diff>
--- a/Agentes.xlsx
+++ b/Agentes.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\000251456\UPBVIRTUAL\Desarrollo\Bots\Agentes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C41790E-2F1E-44B1-B026-03383E8A759A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70CEBB0E-0F64-4CDF-AA51-8EA1A771BA46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DE163BBC-0BFD-48AC-9D42-2B7A41334F44}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{DE163BBC-0BFD-48AC-9D42-2B7A41334F44}"/>
   </bookViews>
   <sheets>
-    <sheet name="Agentes" sheetId="2" r:id="rId1"/>
+    <sheet name="Agentes" sheetId="4" r:id="rId1"/>
     <sheet name="AgentesCONTAR" sheetId="3" r:id="rId2"/>
   </sheets>
   <definedNames>
@@ -437,8 +437,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C55F7F1-5C0E-46A4-B802-59D39193FA07}">
-  <dimension ref="A1:E7"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAD0E336-FF72-4949-B91A-06BB84E75F41}">
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.85546875" customWidth="1"/>
@@ -465,110 +465,875 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>54161</v>
+        <v>51697</v>
       </c>
       <c r="B2">
-        <v>76381</v>
+        <v>80902</v>
       </c>
       <c r="C2">
-        <v>22482</v>
+        <v>24962</v>
       </c>
       <c r="D2" s="1">
-        <v>46007</v>
+        <v>46125</v>
       </c>
       <c r="E2" s="1">
-        <v>46011</v>
+        <v>46166</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>54161</v>
+        <v>51697</v>
       </c>
       <c r="B3">
-        <v>76381</v>
+        <v>80902</v>
       </c>
       <c r="C3">
-        <v>22483</v>
+        <v>24963</v>
       </c>
       <c r="D3" s="1">
-        <v>46007</v>
+        <v>46125</v>
       </c>
       <c r="E3" s="1">
-        <v>46011</v>
+        <v>46166</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>54161</v>
+        <v>51697</v>
       </c>
       <c r="B4">
-        <v>76381</v>
+        <v>80902</v>
       </c>
       <c r="C4">
-        <v>22484</v>
+        <v>24964</v>
       </c>
       <c r="D4" s="1">
-        <v>46007</v>
+        <v>46125</v>
       </c>
       <c r="E4" s="1">
-        <v>46011</v>
+        <v>46166</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>54413</v>
+        <v>30456</v>
       </c>
       <c r="B5">
-        <v>77361</v>
+        <v>82011</v>
       </c>
       <c r="C5">
-        <v>23061</v>
+        <v>25832</v>
       </c>
       <c r="D5" s="1">
-        <v>46007</v>
+        <v>46118</v>
       </c>
       <c r="E5" s="1">
-        <v>46035</v>
+        <v>46187</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>54413</v>
+        <v>30456</v>
       </c>
       <c r="B6">
-        <v>77361</v>
+        <v>82011</v>
       </c>
       <c r="C6">
-        <v>23062</v>
+        <v>25833</v>
       </c>
       <c r="D6" s="1">
-        <v>46007</v>
+        <v>46118</v>
       </c>
       <c r="E6" s="1">
-        <v>46035</v>
+        <v>46187</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>54413</v>
+        <v>30456</v>
       </c>
       <c r="B7">
-        <v>77361</v>
+        <v>82011</v>
       </c>
       <c r="C7">
-        <v>23063</v>
+        <v>25834</v>
       </c>
       <c r="D7" s="1">
-        <v>46007</v>
+        <v>46118</v>
       </c>
       <c r="E7" s="1">
-        <v>46035</v>
+        <v>46187</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>51860</v>
+      </c>
+      <c r="B8">
+        <v>82035</v>
+      </c>
+      <c r="C8">
+        <v>25850</v>
+      </c>
+      <c r="D8" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E8" s="1">
+        <v>46145</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>51860</v>
+      </c>
+      <c r="B9">
+        <v>82035</v>
+      </c>
+      <c r="C9">
+        <v>25851</v>
+      </c>
+      <c r="D9" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E9" s="1">
+        <v>46145</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>51860</v>
+      </c>
+      <c r="B10">
+        <v>82035</v>
+      </c>
+      <c r="C10">
+        <v>25852</v>
+      </c>
+      <c r="D10" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E10" s="1">
+        <v>46145</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>51673</v>
+      </c>
+      <c r="B11">
+        <v>82054</v>
+      </c>
+      <c r="C11">
+        <v>25468</v>
+      </c>
+      <c r="D11" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E11" s="1">
+        <v>46159</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>51673</v>
+      </c>
+      <c r="B12">
+        <v>82054</v>
+      </c>
+      <c r="C12">
+        <v>25469</v>
+      </c>
+      <c r="D12" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E12" s="1">
+        <v>46159</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>51673</v>
+      </c>
+      <c r="B13">
+        <v>82054</v>
+      </c>
+      <c r="C13">
+        <v>25470</v>
+      </c>
+      <c r="D13" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E13" s="1">
+        <v>46159</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>52201</v>
+      </c>
+      <c r="B14">
+        <v>82119</v>
+      </c>
+      <c r="C14">
+        <v>25513</v>
+      </c>
+      <c r="D14" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E14" s="1">
+        <v>46145</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>52201</v>
+      </c>
+      <c r="B15">
+        <v>82119</v>
+      </c>
+      <c r="C15">
+        <v>25514</v>
+      </c>
+      <c r="D15" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E15" s="1">
+        <v>46145</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>52201</v>
+      </c>
+      <c r="B16">
+        <v>82119</v>
+      </c>
+      <c r="C16">
+        <v>25515</v>
+      </c>
+      <c r="D16" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E16" s="1">
+        <v>46145</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>51707</v>
+      </c>
+      <c r="B17">
+        <v>82130</v>
+      </c>
+      <c r="C17">
+        <v>25519</v>
+      </c>
+      <c r="D17" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E17" s="1">
+        <v>46165</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>51707</v>
+      </c>
+      <c r="B18">
+        <v>82130</v>
+      </c>
+      <c r="C18">
+        <v>25520</v>
+      </c>
+      <c r="D18" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E18" s="1">
+        <v>46165</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>51707</v>
+      </c>
+      <c r="B19">
+        <v>82130</v>
+      </c>
+      <c r="C19">
+        <v>25521</v>
+      </c>
+      <c r="D19" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E19" s="1">
+        <v>46165</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>31509</v>
+      </c>
+      <c r="B20">
+        <v>82138</v>
+      </c>
+      <c r="C20">
+        <v>25522</v>
+      </c>
+      <c r="D20" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E20" s="1">
+        <v>46165</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>31509</v>
+      </c>
+      <c r="B21">
+        <v>82138</v>
+      </c>
+      <c r="C21">
+        <v>25523</v>
+      </c>
+      <c r="D21" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E21" s="1">
+        <v>46165</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>31509</v>
+      </c>
+      <c r="B22">
+        <v>82138</v>
+      </c>
+      <c r="C22">
+        <v>25524</v>
+      </c>
+      <c r="D22" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E22" s="1">
+        <v>46165</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>58046</v>
+      </c>
+      <c r="B23">
+        <v>82162</v>
+      </c>
+      <c r="C23">
+        <v>25531</v>
+      </c>
+      <c r="D23" s="1">
+        <v>46123</v>
+      </c>
+      <c r="E23" s="1">
+        <v>46145</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>58046</v>
+      </c>
+      <c r="B24">
+        <v>82162</v>
+      </c>
+      <c r="C24">
+        <v>25532</v>
+      </c>
+      <c r="D24" s="1">
+        <v>46123</v>
+      </c>
+      <c r="E24" s="1">
+        <v>46145</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>58046</v>
+      </c>
+      <c r="B25">
+        <v>82162</v>
+      </c>
+      <c r="C25">
+        <v>25533</v>
+      </c>
+      <c r="D25" s="1">
+        <v>46123</v>
+      </c>
+      <c r="E25" s="1">
+        <v>46145</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>52253</v>
+      </c>
+      <c r="B26">
+        <v>82205</v>
+      </c>
+      <c r="C26">
+        <v>25540</v>
+      </c>
+      <c r="D26" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E26" s="1">
+        <v>46148</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>52253</v>
+      </c>
+      <c r="B27">
+        <v>82205</v>
+      </c>
+      <c r="C27">
+        <v>25541</v>
+      </c>
+      <c r="D27" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E27" s="1">
+        <v>46148</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>52253</v>
+      </c>
+      <c r="B28">
+        <v>82205</v>
+      </c>
+      <c r="C28">
+        <v>25542</v>
+      </c>
+      <c r="D28" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E28" s="1">
+        <v>46148</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>51407</v>
+      </c>
+      <c r="B29">
+        <v>82212</v>
+      </c>
+      <c r="C29">
+        <v>25543</v>
+      </c>
+      <c r="D29" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E29" s="1">
+        <v>46144</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>51407</v>
+      </c>
+      <c r="B30">
+        <v>82212</v>
+      </c>
+      <c r="C30">
+        <v>25544</v>
+      </c>
+      <c r="D30" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E30" s="1">
+        <v>46144</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>51407</v>
+      </c>
+      <c r="B31">
+        <v>82212</v>
+      </c>
+      <c r="C31">
+        <v>25545</v>
+      </c>
+      <c r="D31" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E31" s="1">
+        <v>46144</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>51440</v>
+      </c>
+      <c r="B32">
+        <v>82231</v>
+      </c>
+      <c r="C32">
+        <v>25549</v>
+      </c>
+      <c r="D32" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E32" s="1">
+        <v>46144</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>51440</v>
+      </c>
+      <c r="B33">
+        <v>82231</v>
+      </c>
+      <c r="C33">
+        <v>25550</v>
+      </c>
+      <c r="D33" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E33" s="1">
+        <v>46144</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>51440</v>
+      </c>
+      <c r="B34">
+        <v>82231</v>
+      </c>
+      <c r="C34">
+        <v>25551</v>
+      </c>
+      <c r="D34" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E34" s="1">
+        <v>46144</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>51447</v>
+      </c>
+      <c r="B35">
+        <v>82238</v>
+      </c>
+      <c r="C35">
+        <v>25555</v>
+      </c>
+      <c r="D35" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E35" s="1">
+        <v>46144</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>51447</v>
+      </c>
+      <c r="B36">
+        <v>82238</v>
+      </c>
+      <c r="C36">
+        <v>25556</v>
+      </c>
+      <c r="D36" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E36" s="1">
+        <v>46144</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>51447</v>
+      </c>
+      <c r="B37">
+        <v>82238</v>
+      </c>
+      <c r="C37">
+        <v>25557</v>
+      </c>
+      <c r="D37" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E37" s="1">
+        <v>46144</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>51176</v>
+      </c>
+      <c r="B38">
+        <v>82253</v>
+      </c>
+      <c r="C38">
+        <v>25561</v>
+      </c>
+      <c r="D38" s="1">
+        <v>46127</v>
+      </c>
+      <c r="E38" s="1">
+        <v>46191</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>51176</v>
+      </c>
+      <c r="B39">
+        <v>82253</v>
+      </c>
+      <c r="C39">
+        <v>25562</v>
+      </c>
+      <c r="D39" s="1">
+        <v>46127</v>
+      </c>
+      <c r="E39" s="1">
+        <v>46191</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>51176</v>
+      </c>
+      <c r="B40">
+        <v>82253</v>
+      </c>
+      <c r="C40">
+        <v>25563</v>
+      </c>
+      <c r="D40" s="1">
+        <v>46127</v>
+      </c>
+      <c r="E40" s="1">
+        <v>46191</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>50674</v>
+      </c>
+      <c r="B41">
+        <v>82926</v>
+      </c>
+      <c r="C41">
+        <v>25781</v>
+      </c>
+      <c r="D41" s="1">
+        <v>46118</v>
+      </c>
+      <c r="E41" s="1">
+        <v>46172</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>50674</v>
+      </c>
+      <c r="B42">
+        <v>82926</v>
+      </c>
+      <c r="C42">
+        <v>25782</v>
+      </c>
+      <c r="D42" s="1">
+        <v>46118</v>
+      </c>
+      <c r="E42" s="1">
+        <v>46172</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>50674</v>
+      </c>
+      <c r="B43">
+        <v>82926</v>
+      </c>
+      <c r="C43">
+        <v>25783</v>
+      </c>
+      <c r="D43" s="1">
+        <v>46118</v>
+      </c>
+      <c r="E43" s="1">
+        <v>46172</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>52410</v>
+      </c>
+      <c r="B44">
+        <v>83116</v>
+      </c>
+      <c r="C44">
+        <v>25841</v>
+      </c>
+      <c r="D44" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E44" s="1">
+        <v>46185</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>52410</v>
+      </c>
+      <c r="B45">
+        <v>83116</v>
+      </c>
+      <c r="C45">
+        <v>25842</v>
+      </c>
+      <c r="D45" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E45" s="1">
+        <v>46185</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>52410</v>
+      </c>
+      <c r="B46">
+        <v>83116</v>
+      </c>
+      <c r="C46">
+        <v>25843</v>
+      </c>
+      <c r="D46" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E46" s="1">
+        <v>46185</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47" s="2">
+        <v>51742</v>
+      </c>
+      <c r="B47">
+        <v>83127</v>
+      </c>
+      <c r="C47">
+        <v>25844</v>
+      </c>
+      <c r="D47" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E47" s="1">
+        <v>46189</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" s="2">
+        <v>51742</v>
+      </c>
+      <c r="B48">
+        <v>83127</v>
+      </c>
+      <c r="C48">
+        <v>25845</v>
+      </c>
+      <c r="D48" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E48" s="1">
+        <v>46189</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" s="2">
+        <v>51742</v>
+      </c>
+      <c r="B49">
+        <v>83127</v>
+      </c>
+      <c r="C49">
+        <v>25846</v>
+      </c>
+      <c r="D49" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E49" s="1">
+        <v>46189</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" s="2">
+        <v>51948</v>
+      </c>
+      <c r="B50">
+        <v>83144</v>
+      </c>
+      <c r="C50">
+        <v>25853</v>
+      </c>
+      <c r="D50" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E50" s="1">
+        <v>46152</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" s="2">
+        <v>51948</v>
+      </c>
+      <c r="B51">
+        <v>83144</v>
+      </c>
+      <c r="C51">
+        <v>25854</v>
+      </c>
+      <c r="D51" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E51" s="1">
+        <v>46152</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" s="2">
+        <v>51948</v>
+      </c>
+      <c r="B52">
+        <v>83144</v>
+      </c>
+      <c r="C52">
+        <v>25855</v>
+      </c>
+      <c r="D52" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E52" s="1">
+        <v>46152</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:E1" xr:uid="{7C55F7F1-5C0E-46A4-B802-59D39193FA07}"/>
   <conditionalFormatting sqref="B1:B1048576">
-    <cfRule type="duplicateValues" dxfId="0" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -577,7 +1342,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24AF5C5D-7673-444A-AA6F-420E0326BAC3}">
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.85546875" customWidth="1"/>
@@ -629,40 +1394,40 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>54161</v>
+        <v>51697</v>
       </c>
       <c r="B3">
-        <v>76381</v>
+        <v>80902</v>
       </c>
       <c r="C3">
-        <v>22482</v>
+        <v>24962</v>
       </c>
       <c r="D3" s="1">
-        <v>46007</v>
+        <v>46125</v>
       </c>
       <c r="E3" s="1">
-        <v>46011</v>
+        <v>46166</v>
       </c>
       <c r="F3" s="2">
-        <f t="shared" ref="F3:F8" si="0">COUNTIFS(B:B,B3)</f>
+        <f t="shared" ref="F3:F53" si="0">COUNTIFS(B:B,B3)</f>
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>54161</v>
+        <v>51697</v>
       </c>
       <c r="B4">
-        <v>76381</v>
+        <v>80902</v>
       </c>
       <c r="C4">
-        <v>22483</v>
+        <v>24963</v>
       </c>
       <c r="D4" s="1">
-        <v>46007</v>
+        <v>46125</v>
       </c>
       <c r="E4" s="1">
-        <v>46011</v>
+        <v>46166</v>
       </c>
       <c r="F4" s="2">
         <f t="shared" si="0"/>
@@ -671,19 +1436,19 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>54161</v>
+        <v>51697</v>
       </c>
       <c r="B5">
-        <v>76381</v>
+        <v>80902</v>
       </c>
       <c r="C5">
-        <v>22484</v>
+        <v>24964</v>
       </c>
       <c r="D5" s="1">
-        <v>46007</v>
+        <v>46125</v>
       </c>
       <c r="E5" s="1">
-        <v>46011</v>
+        <v>46166</v>
       </c>
       <c r="F5" s="2">
         <f t="shared" si="0"/>
@@ -692,19 +1457,19 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>54413</v>
+        <v>30456</v>
       </c>
       <c r="B6">
-        <v>77361</v>
+        <v>82011</v>
       </c>
       <c r="C6">
-        <v>23061</v>
+        <v>25832</v>
       </c>
       <c r="D6" s="1">
-        <v>46007</v>
+        <v>46118</v>
       </c>
       <c r="E6" s="1">
-        <v>46035</v>
+        <v>46187</v>
       </c>
       <c r="F6" s="2">
         <f t="shared" si="0"/>
@@ -713,19 +1478,19 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>54413</v>
+        <v>30456</v>
       </c>
       <c r="B7">
-        <v>77361</v>
+        <v>82011</v>
       </c>
       <c r="C7">
-        <v>23062</v>
+        <v>25833</v>
       </c>
       <c r="D7" s="1">
-        <v>46007</v>
+        <v>46118</v>
       </c>
       <c r="E7" s="1">
-        <v>46035</v>
+        <v>46187</v>
       </c>
       <c r="F7" s="2">
         <f t="shared" si="0"/>
@@ -734,21 +1499,966 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>54413</v>
+        <v>30456</v>
       </c>
       <c r="B8">
-        <v>77361</v>
+        <v>82011</v>
       </c>
       <c r="C8">
-        <v>23063</v>
+        <v>25834</v>
       </c>
       <c r="D8" s="1">
-        <v>46007</v>
+        <v>46118</v>
       </c>
       <c r="E8" s="1">
-        <v>46035</v>
+        <v>46187</v>
       </c>
       <c r="F8" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>51860</v>
+      </c>
+      <c r="B9">
+        <v>82035</v>
+      </c>
+      <c r="C9">
+        <v>25850</v>
+      </c>
+      <c r="D9" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E9" s="1">
+        <v>46145</v>
+      </c>
+      <c r="F9" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>51860</v>
+      </c>
+      <c r="B10">
+        <v>82035</v>
+      </c>
+      <c r="C10">
+        <v>25851</v>
+      </c>
+      <c r="D10" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E10" s="1">
+        <v>46145</v>
+      </c>
+      <c r="F10" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>51860</v>
+      </c>
+      <c r="B11">
+        <v>82035</v>
+      </c>
+      <c r="C11">
+        <v>25852</v>
+      </c>
+      <c r="D11" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E11" s="1">
+        <v>46145</v>
+      </c>
+      <c r="F11" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>51673</v>
+      </c>
+      <c r="B12">
+        <v>82054</v>
+      </c>
+      <c r="C12">
+        <v>25468</v>
+      </c>
+      <c r="D12" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E12" s="1">
+        <v>46159</v>
+      </c>
+      <c r="F12" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>51673</v>
+      </c>
+      <c r="B13">
+        <v>82054</v>
+      </c>
+      <c r="C13">
+        <v>25469</v>
+      </c>
+      <c r="D13" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E13" s="1">
+        <v>46159</v>
+      </c>
+      <c r="F13" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>51673</v>
+      </c>
+      <c r="B14">
+        <v>82054</v>
+      </c>
+      <c r="C14">
+        <v>25470</v>
+      </c>
+      <c r="D14" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E14" s="1">
+        <v>46159</v>
+      </c>
+      <c r="F14" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>52201</v>
+      </c>
+      <c r="B15">
+        <v>82119</v>
+      </c>
+      <c r="C15">
+        <v>25513</v>
+      </c>
+      <c r="D15" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E15" s="1">
+        <v>46145</v>
+      </c>
+      <c r="F15" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>52201</v>
+      </c>
+      <c r="B16">
+        <v>82119</v>
+      </c>
+      <c r="C16">
+        <v>25514</v>
+      </c>
+      <c r="D16" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E16" s="1">
+        <v>46145</v>
+      </c>
+      <c r="F16" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>52201</v>
+      </c>
+      <c r="B17">
+        <v>82119</v>
+      </c>
+      <c r="C17">
+        <v>25515</v>
+      </c>
+      <c r="D17" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E17" s="1">
+        <v>46145</v>
+      </c>
+      <c r="F17" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>51707</v>
+      </c>
+      <c r="B18">
+        <v>82130</v>
+      </c>
+      <c r="C18">
+        <v>25519</v>
+      </c>
+      <c r="D18" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E18" s="1">
+        <v>46165</v>
+      </c>
+      <c r="F18" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>51707</v>
+      </c>
+      <c r="B19">
+        <v>82130</v>
+      </c>
+      <c r="C19">
+        <v>25520</v>
+      </c>
+      <c r="D19" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E19" s="1">
+        <v>46165</v>
+      </c>
+      <c r="F19" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>51707</v>
+      </c>
+      <c r="B20">
+        <v>82130</v>
+      </c>
+      <c r="C20">
+        <v>25521</v>
+      </c>
+      <c r="D20" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E20" s="1">
+        <v>46165</v>
+      </c>
+      <c r="F20" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>31509</v>
+      </c>
+      <c r="B21">
+        <v>82138</v>
+      </c>
+      <c r="C21">
+        <v>25522</v>
+      </c>
+      <c r="D21" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E21" s="1">
+        <v>46165</v>
+      </c>
+      <c r="F21" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>31509</v>
+      </c>
+      <c r="B22">
+        <v>82138</v>
+      </c>
+      <c r="C22">
+        <v>25523</v>
+      </c>
+      <c r="D22" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E22" s="1">
+        <v>46165</v>
+      </c>
+      <c r="F22" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>31509</v>
+      </c>
+      <c r="B23">
+        <v>82138</v>
+      </c>
+      <c r="C23">
+        <v>25524</v>
+      </c>
+      <c r="D23" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E23" s="1">
+        <v>46165</v>
+      </c>
+      <c r="F23" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>58046</v>
+      </c>
+      <c r="B24">
+        <v>82162</v>
+      </c>
+      <c r="C24">
+        <v>25531</v>
+      </c>
+      <c r="D24" s="1">
+        <v>46123</v>
+      </c>
+      <c r="E24" s="1">
+        <v>46145</v>
+      </c>
+      <c r="F24" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>58046</v>
+      </c>
+      <c r="B25">
+        <v>82162</v>
+      </c>
+      <c r="C25">
+        <v>25532</v>
+      </c>
+      <c r="D25" s="1">
+        <v>46123</v>
+      </c>
+      <c r="E25" s="1">
+        <v>46145</v>
+      </c>
+      <c r="F25" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>58046</v>
+      </c>
+      <c r="B26">
+        <v>82162</v>
+      </c>
+      <c r="C26">
+        <v>25533</v>
+      </c>
+      <c r="D26" s="1">
+        <v>46123</v>
+      </c>
+      <c r="E26" s="1">
+        <v>46145</v>
+      </c>
+      <c r="F26" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>52253</v>
+      </c>
+      <c r="B27">
+        <v>82205</v>
+      </c>
+      <c r="C27">
+        <v>25540</v>
+      </c>
+      <c r="D27" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E27" s="1">
+        <v>46148</v>
+      </c>
+      <c r="F27" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>52253</v>
+      </c>
+      <c r="B28">
+        <v>82205</v>
+      </c>
+      <c r="C28">
+        <v>25541</v>
+      </c>
+      <c r="D28" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E28" s="1">
+        <v>46148</v>
+      </c>
+      <c r="F28" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>52253</v>
+      </c>
+      <c r="B29">
+        <v>82205</v>
+      </c>
+      <c r="C29">
+        <v>25542</v>
+      </c>
+      <c r="D29" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E29" s="1">
+        <v>46148</v>
+      </c>
+      <c r="F29" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>51407</v>
+      </c>
+      <c r="B30">
+        <v>82212</v>
+      </c>
+      <c r="C30">
+        <v>25543</v>
+      </c>
+      <c r="D30" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E30" s="1">
+        <v>46144</v>
+      </c>
+      <c r="F30" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>51407</v>
+      </c>
+      <c r="B31">
+        <v>82212</v>
+      </c>
+      <c r="C31">
+        <v>25544</v>
+      </c>
+      <c r="D31" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E31" s="1">
+        <v>46144</v>
+      </c>
+      <c r="F31" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>51407</v>
+      </c>
+      <c r="B32">
+        <v>82212</v>
+      </c>
+      <c r="C32">
+        <v>25545</v>
+      </c>
+      <c r="D32" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E32" s="1">
+        <v>46144</v>
+      </c>
+      <c r="F32" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>51440</v>
+      </c>
+      <c r="B33">
+        <v>82231</v>
+      </c>
+      <c r="C33">
+        <v>25549</v>
+      </c>
+      <c r="D33" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E33" s="1">
+        <v>46144</v>
+      </c>
+      <c r="F33" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>51440</v>
+      </c>
+      <c r="B34">
+        <v>82231</v>
+      </c>
+      <c r="C34">
+        <v>25550</v>
+      </c>
+      <c r="D34" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E34" s="1">
+        <v>46144</v>
+      </c>
+      <c r="F34" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>51440</v>
+      </c>
+      <c r="B35">
+        <v>82231</v>
+      </c>
+      <c r="C35">
+        <v>25551</v>
+      </c>
+      <c r="D35" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E35" s="1">
+        <v>46144</v>
+      </c>
+      <c r="F35" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>51447</v>
+      </c>
+      <c r="B36">
+        <v>82238</v>
+      </c>
+      <c r="C36">
+        <v>25555</v>
+      </c>
+      <c r="D36" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E36" s="1">
+        <v>46144</v>
+      </c>
+      <c r="F36" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>51447</v>
+      </c>
+      <c r="B37">
+        <v>82238</v>
+      </c>
+      <c r="C37">
+        <v>25556</v>
+      </c>
+      <c r="D37" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E37" s="1">
+        <v>46144</v>
+      </c>
+      <c r="F37" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>51447</v>
+      </c>
+      <c r="B38">
+        <v>82238</v>
+      </c>
+      <c r="C38">
+        <v>25557</v>
+      </c>
+      <c r="D38" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E38" s="1">
+        <v>46144</v>
+      </c>
+      <c r="F38" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>51176</v>
+      </c>
+      <c r="B39">
+        <v>82253</v>
+      </c>
+      <c r="C39">
+        <v>25561</v>
+      </c>
+      <c r="D39" s="1">
+        <v>46127</v>
+      </c>
+      <c r="E39" s="1">
+        <v>46191</v>
+      </c>
+      <c r="F39" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>51176</v>
+      </c>
+      <c r="B40">
+        <v>82253</v>
+      </c>
+      <c r="C40">
+        <v>25562</v>
+      </c>
+      <c r="D40" s="1">
+        <v>46127</v>
+      </c>
+      <c r="E40" s="1">
+        <v>46191</v>
+      </c>
+      <c r="F40" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>51176</v>
+      </c>
+      <c r="B41">
+        <v>82253</v>
+      </c>
+      <c r="C41">
+        <v>25563</v>
+      </c>
+      <c r="D41" s="1">
+        <v>46127</v>
+      </c>
+      <c r="E41" s="1">
+        <v>46191</v>
+      </c>
+      <c r="F41" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>50674</v>
+      </c>
+      <c r="B42">
+        <v>82926</v>
+      </c>
+      <c r="C42">
+        <v>25781</v>
+      </c>
+      <c r="D42" s="1">
+        <v>46118</v>
+      </c>
+      <c r="E42" s="1">
+        <v>46172</v>
+      </c>
+      <c r="F42" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>50674</v>
+      </c>
+      <c r="B43">
+        <v>82926</v>
+      </c>
+      <c r="C43">
+        <v>25782</v>
+      </c>
+      <c r="D43" s="1">
+        <v>46118</v>
+      </c>
+      <c r="E43" s="1">
+        <v>46172</v>
+      </c>
+      <c r="F43" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>50674</v>
+      </c>
+      <c r="B44">
+        <v>82926</v>
+      </c>
+      <c r="C44">
+        <v>25783</v>
+      </c>
+      <c r="D44" s="1">
+        <v>46118</v>
+      </c>
+      <c r="E44" s="1">
+        <v>46172</v>
+      </c>
+      <c r="F44" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>52410</v>
+      </c>
+      <c r="B45">
+        <v>83116</v>
+      </c>
+      <c r="C45">
+        <v>25841</v>
+      </c>
+      <c r="D45" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E45" s="1">
+        <v>46185</v>
+      </c>
+      <c r="F45" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>52410</v>
+      </c>
+      <c r="B46">
+        <v>83116</v>
+      </c>
+      <c r="C46">
+        <v>25842</v>
+      </c>
+      <c r="D46" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E46" s="1">
+        <v>46185</v>
+      </c>
+      <c r="F46" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47">
+        <v>52410</v>
+      </c>
+      <c r="B47">
+        <v>83116</v>
+      </c>
+      <c r="C47">
+        <v>25843</v>
+      </c>
+      <c r="D47" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E47" s="1">
+        <v>46185</v>
+      </c>
+      <c r="F47" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>51742</v>
+      </c>
+      <c r="B48">
+        <v>83127</v>
+      </c>
+      <c r="C48">
+        <v>25844</v>
+      </c>
+      <c r="D48" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E48" s="1">
+        <v>46189</v>
+      </c>
+      <c r="F48" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>51742</v>
+      </c>
+      <c r="B49">
+        <v>83127</v>
+      </c>
+      <c r="C49">
+        <v>25845</v>
+      </c>
+      <c r="D49" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E49" s="1">
+        <v>46189</v>
+      </c>
+      <c r="F49" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <v>51742</v>
+      </c>
+      <c r="B50">
+        <v>83127</v>
+      </c>
+      <c r="C50">
+        <v>25846</v>
+      </c>
+      <c r="D50" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E50" s="1">
+        <v>46189</v>
+      </c>
+      <c r="F50" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>51948</v>
+      </c>
+      <c r="B51">
+        <v>83144</v>
+      </c>
+      <c r="C51">
+        <v>25853</v>
+      </c>
+      <c r="D51" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E51" s="1">
+        <v>46152</v>
+      </c>
+      <c r="F51" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>51948</v>
+      </c>
+      <c r="B52">
+        <v>83144</v>
+      </c>
+      <c r="C52">
+        <v>25854</v>
+      </c>
+      <c r="D52" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E52" s="1">
+        <v>46152</v>
+      </c>
+      <c r="F52" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>51948</v>
+      </c>
+      <c r="B53">
+        <v>83144</v>
+      </c>
+      <c r="C53">
+        <v>25855</v>
+      </c>
+      <c r="D53" s="1">
+        <v>46125</v>
+      </c>
+      <c r="E53" s="1">
+        <v>46152</v>
+      </c>
+      <c r="F53" s="2">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>

</xml_diff>